<commit_message>
Google-Bestaetigung und korrigierte Automaten-Erfahrungswerte
Enes hat die Zahlen aus seiner Praxis gegengelesen und drei korrigiert:
Standortmiete 50-150 EUR statt 0-80, Automat neu 5.000-15.000 statt
3.000-8.000, gebraucht 2.000-4.000 statt 800-2.500. Die alten Werte
waren zu niedrig gegriffen -- ein Praktiker haette sie sofort als
falsch erkannt, und genau diese Leser sollen das Produkt kaufen.

Dazu die Bestaetigungsdatei fuer die Google Search Console, damit die
Seite aktiv angemeldet werden kann statt auf Googles Zufallsbesuch zu
warten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/produkte/Automaten-Rentabilitaetsrechner.xlsx
+++ b/produkte/Automaten-Rentabilitaetsrechner.xlsx
@@ -1950,11 +1950,11 @@
         </is>
       </c>
       <c r="C20" s="35" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>Übliche Spanne 0 bis 80 €. Viele Standorte geben die Fläche umsonst her, wenn der Automat gewünscht ist.</t>
+          <t>Übliche Spanne 50 bis 150 €. Frag trotzdem, ob der Betrieb darauf verzichtet — manche geben die Fläche umsonst her, wenn der Automat gewünscht ist.</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="D54" s="28" t="inlineStr">
         <is>
-          <t>Gebraucht 800–2.500 €, neu 3.000–8.000 €. Bei Miete oder Leasing hier 0 eintragen und die Rate unter „Sonstiges“ erfassen.</t>
+          <t>Gebraucht 2.000–4.000 €, neu 5.000–15.000 €. Bei Miete oder Leasing hier 0 eintragen und die Rate unter „Sonstiges“ erfassen.</t>
         </is>
       </c>
     </row>
@@ -2962,12 +2962,12 @@
       </c>
       <c r="C8" s="51" t="inlineStr">
         <is>
-          <t>0 – 80 € / Monat</t>
+          <t>50 – 150 € / Monat</t>
         </is>
       </c>
       <c r="D8" s="51" t="inlineStr">
         <is>
-          <t>Viele Betriebe verlangen nichts, wenn die Belegschaft den Automaten will. Immer zuerst nach der kostenlosen Variante fragen.</t>
+          <t>Frag trotzdem zuerst, ob der Betrieb auf die Miete verzichtet — manche tun das, wenn die Belegschaft den Automaten selbst will.</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="C12" s="51" t="inlineStr">
         <is>
-          <t>800 – 2.500 €</t>
+          <t>2.000 – 4.000 €, im Einzelfall mehr</t>
         </is>
       </c>
       <c r="D12" s="51" t="inlineStr">
         <is>
-          <t>Auf Ersatzteilversorgung und Münzprüfer achten. Ein Gerät ohne Ersatzteile ist beim ersten Defekt Schrott.</t>
+          <t>Junge Geräte mit Kühlung und Kartenzahlung liegen deutlich darüber. Auf Ersatzteilversorgung und Münzprüfer achten: ein Gerät ohne Ersatzteile ist beim ersten Defekt Schrott.</t>
         </is>
       </c>
     </row>
@@ -3047,12 +3047,12 @@
       </c>
       <c r="C13" s="51" t="inlineStr">
         <is>
-          <t>3.000 – 8.000 €</t>
+          <t>5.000 – 15.000 €</t>
         </is>
       </c>
       <c r="D13" s="51" t="inlineStr">
         <is>
-          <t>Rechnet sich meist erst ab mehreren Standorten oder bei Kartenzahlung.</t>
+          <t>Die Spanne ist groß: ein einfacher Spiralautomat liegt unten, ein Kombigerät mit Kühlung und Kartenzahlung oben.</t>
         </is>
       </c>
     </row>

</xml_diff>